<commit_message>
feat: OneBot 11 接入模块（Phase 1）
- lib/onebot/client.mjs：正向 WS 客户端，状态机显式建模（含迁移流水）、
  echo 关联 API 调用（超时兜底）、指数退避重连、心跳半死检测、脏数据容错
- lib/onebot/events.mjs：事件归一化（camelCase 内部契约）+ CQ 消息构造
- 错误码体系：EBOT-NOT-CONNECTED / EBOT-API-TIMEOUT / EBOT-DISPOSED / EBOT-API-<retcode> / EBOT-SEND-FAILED / EBOT-BAD-MESSAGE
- 12 个新测试（mock NapCat ws 服务器），全套 39 个测试通过
- 测试用例 Excel 更新至 34 条
</commit_message>
<xml_diff>
--- a/docs/test-cases.xlsx
+++ b/docs/test-cases.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1173,6 +1173,492 @@
       </c>
       <c r="G21" s="2" t="inlineStr"/>
     </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>TC-OB-001</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>OneBot</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>连接建立</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>NapCat 正向 WS 可用</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>start()</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>状态机 disconnected→connecting→connected；生命周期事件不报错</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>TC-OB-002</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>OneBot</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>私聊消息归一化</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>已连接</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>收到 private message 包</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>事件 {type:message, subType:private, userId, text, senderName} 各字段正确</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>TC-OB-003</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>OneBot</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>群消息归一化</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>已连接</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>收到 group message 包</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>groupId/群名片正确；表情等非文本段原样保留在 segments</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>TC-OB-004</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>OneBot</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>API 调用成功</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>已连接</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>callApi(send_private_msg)</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>resolve 为响应 data 字段（如 message_id）</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>TC-OB-005</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>OneBot</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>API 调用失败</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>已连接</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>服务端回 status=failed retcode=1403</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>reject 带 EBOT-API-1403 与错误文案</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>EBOT-API-1403</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>TC-OB-006</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>OneBot</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>API 超时</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>服务器收到请求但不回包</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>callApi（超时阈值 80ms）</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>reject EBOT-API-TIMEOUT</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>EBOT-API-TIMEOUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>TC-OB-007</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>OneBot</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>未连接时调用 API</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>客户端从未 start()</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>callApi</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>立即 reject EBOT-NOT-CONNECTED，不傻等</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>EBOT-NOT-CONNECTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>TC-OB-008</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>OneBot</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>断线自动重连</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>连接被服务端主动断开</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>等待重连</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>状态经 reconnecting 回到 connected；退避间隔非降且不低于基数</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>TC-OB-009</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>OneBot</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>断线时在途调用</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>有 API 在途未回包时断线</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>服务端掐断连接</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>在途调用立即 reject EBOT-NOT-CONNECTED</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>EBOT-NOT-CONNECTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>TC-OB-010</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>OneBot</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>dispose 终态</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>任意运行状态</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>dispose()</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>状态=disposed；不再重连；新调用 reject EBOT-DISPOSED</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>EBOT-DISPOSED</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>TC-OB-011</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>OneBot</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>脏数据容错</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>连接收到非 JSON 包</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>继续收发消息</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>坏包被忽略记日志；连接不崩；后续正常事件照常处理</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>TC-OB-012</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>OneBot</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>处理器异常隔离</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>某个事件处理器抛异常</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>继续分发事件</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>其他处理器照常收到事件；连接不断</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>TC-OB-013</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>OneBot</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>access_token 传递</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>配置 onebot.token</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>建立连接</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>NapCat 侧收到的 URL 带 access_token=&lt;token&gt;</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>TC-OB-014</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>OneBot</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>回复消息构造契约</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>buildMessage(文本/对象/数组/数字)</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>CQ 段输出符合契约；非法输入抛 EBOT-BAD-MESSAGE</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>EBOT-BAD-MESSAGE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>